<commit_message>
Trektellen exports refreshed to 12 October 2026, with the new days' survey status
The 2026 export adds 2-12 October (3,337 rows). In 2024 one record's name
changes (redpoll sp. -> Redpoll) and the header gains hpa and hydro; in
2025 LPO 74 corrected survey stop times upstream on 13 October (one had
ended at 05:50 the next morning). 2023 and the 2025 counts are unchanged
in content.

Survey status: the 1 October weather stop bounded by the recorded end,
the 7 October weather stops, and 3595350 reviewed as continuous counting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/trektellen/Trektellen_headerdata_2422_2025.xlsx
+++ b/raw/trektellen/Trektellen_headerdata_2422_2025.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="828">
   <si>
     <t>id</t>
   </si>
@@ -782,7 +782,7 @@
     <t>2025-08-24 06:43:00</t>
   </si>
   <si>
-    <t>2025-08-25 05:36:00</t>
+    <t>2025-08-24 20:30:00</t>
   </si>
   <si>
     <t xml:space="preserve">Dominique Maire, Sati Boulicot, Pascal Charrière, Lutz Lucker, Gras Michel, Frédérique Dalla-Libera, Christine Chaban, Martinet Michel-Passagury, Bernard Monnier </t>
@@ -800,6 +800,9 @@
     <t>2026-03-11 14:57:46.090219</t>
   </si>
   <si>
+    <t>2026-10-13 09:01:35.713825</t>
+  </si>
+  <si>
     <t>2025-08-25 06:48:00</t>
   </si>
   <si>
@@ -1034,10 +1037,10 @@
     <t>2025-09-07 06:56:00</t>
   </si>
   <si>
-    <t>2025-09-08 05:56:00</t>
-  </si>
-  <si>
-    <t>Dominique Maire, Thibault Goutin (avec formation LPO 74), Groupe jeune "nos oiseaux"(Suisse), Clément Sittler, Frédérique et Michel Gras, Catherine Dombray, Sylvie Mas, Pierre Rebelle, Michel Faure, Stéphane Henneberg</t>
+    <t>2025-09-07 20:02:00</t>
+  </si>
+  <si>
+    <t>Dominique Maire, Thibault Goutin (avec formation LPO 74), Groupe jeune &amp;quot;nos oiseaux&amp;quot;(Suisse), Clément Sittler, Frédérique et Michel Gras, Catherine Dombray, Sylvie Mas, Pierre Rebelle, Michel Faure, Stéphane Henneberg</t>
   </si>
   <si>
     <t xml:space="preserve">Ciel bleu </t>
@@ -1046,6 +1049,9 @@
     <t>2026-03-11 14:57:45.484501</t>
   </si>
   <si>
+    <t>2026-10-13 09:03:51.495839</t>
+  </si>
+  <si>
     <t>2025-09-08 07:06:00</t>
   </si>
   <si>
@@ -1271,7 +1277,7 @@
     <t>2025-09-21 07:19:00</t>
   </si>
   <si>
-    <t>2025-09-22 06:09:00</t>
+    <t>2025-09-21 19:36:00</t>
   </si>
   <si>
     <t>Dominique Maire, Lutz Lucker et Sylvie Frémont, Valentin Roussel, Claire Dumortier, Michel Gras et Frédérique.</t>
@@ -1289,6 +1295,9 @@
     <t>2026-03-11 14:57:44.25079</t>
   </si>
   <si>
+    <t>2026-10-13 09:04:36.438232</t>
+  </si>
+  <si>
     <t>2025-09-22 07:23:00</t>
   </si>
   <si>
@@ -1769,19 +1778,22 @@
     <t>2025-10-19 07:58:00</t>
   </si>
   <si>
-    <t>2025-10-20 05:50:00</t>
+    <t>2025-10-19 18:44:00</t>
   </si>
   <si>
     <t>Dominique Maire, Michel et Frédérique Gras, Isabelle et Roger Cattin Gasser.</t>
   </si>
   <si>
-    <t>Brouillard une partie de la matinée, puis quelques éclaircies, fin d'après midi très nuageux.</t>
+    <t>Brouillard une partie de la matinée, puis quelques éclaircies, fin d&amp;#039;après midi très nuageux.</t>
   </si>
   <si>
     <t>zw</t>
   </si>
   <si>
     <t>2026-03-11 14:57:41.635804</t>
+  </si>
+  <si>
+    <t>2026-10-13 09:05:40.212079</t>
   </si>
   <si>
     <t>2025-10-20 08:00:00</t>
@@ -5162,7 +5174,10 @@
         <v>37</v>
       </c>
       <c r="AC39" t="s">
-        <v>260</v>
+        <v>261</v>
+      </c>
+      <c r="AD39" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:30">
@@ -5188,13 +5203,13 @@
         <v>2025</v>
       </c>
       <c r="H40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I40" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J40" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P40">
         <v>0</v>
@@ -5209,16 +5224,16 @@
         <v>34</v>
       </c>
       <c r="Z40" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AA40" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AB40" t="s">
         <v>37</v>
       </c>
       <c r="AC40" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AD40" t="s">
         <v>37</v>
@@ -5247,13 +5262,13 @@
         <v>2025</v>
       </c>
       <c r="H41" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I41" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="P41">
         <v>0</v>
@@ -5268,16 +5283,16 @@
         <v>34</v>
       </c>
       <c r="Z41" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AA41" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AB41" t="s">
         <v>37</v>
       </c>
       <c r="AC41" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AD41" t="s">
         <v>37</v>
@@ -5306,13 +5321,13 @@
         <v>2025</v>
       </c>
       <c r="H42" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I42" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J42" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P42">
         <v>0</v>
@@ -5327,16 +5342,16 @@
         <v>34</v>
       </c>
       <c r="Z42" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="AA42" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AB42" t="s">
         <v>37</v>
       </c>
       <c r="AC42" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AD42" t="s">
         <v>37</v>
@@ -5365,13 +5380,13 @@
         <v>2025</v>
       </c>
       <c r="H43" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I43" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J43" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P43">
         <v>0</v>
@@ -5386,16 +5401,16 @@
         <v>34</v>
       </c>
       <c r="Z43" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AA43" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AB43" t="s">
         <v>37</v>
       </c>
       <c r="AC43" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AD43" t="s">
         <v>37</v>
@@ -5424,13 +5439,13 @@
         <v>2025</v>
       </c>
       <c r="H44" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I44" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J44" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P44">
         <v>0</v>
@@ -5445,16 +5460,16 @@
         <v>34</v>
       </c>
       <c r="Z44" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="AA44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="AB44" t="s">
         <v>37</v>
       </c>
       <c r="AC44" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AD44" t="s">
         <v>37</v>
@@ -5483,13 +5498,13 @@
         <v>2025</v>
       </c>
       <c r="H45" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I45" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J45" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="P45">
         <v>0</v>
@@ -5504,16 +5519,16 @@
         <v>34</v>
       </c>
       <c r="Z45" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AA45" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AB45" t="s">
         <v>37</v>
       </c>
       <c r="AC45" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AD45" t="s">
         <v>37</v>
@@ -5542,13 +5557,13 @@
         <v>2025</v>
       </c>
       <c r="H46" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I46" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J46" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P46">
         <v>0</v>
@@ -5569,13 +5584,13 @@
         <v>34</v>
       </c>
       <c r="AA46" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AB46" t="s">
         <v>37</v>
       </c>
       <c r="AC46" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AD46" t="s">
         <v>37</v>
@@ -5604,13 +5619,13 @@
         <v>2025</v>
       </c>
       <c r="H47" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="I47" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J47" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="P47">
         <v>0</v>
@@ -5625,16 +5640,16 @@
         <v>34</v>
       </c>
       <c r="Z47" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AA47" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AB47" t="s">
         <v>37</v>
       </c>
       <c r="AC47" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AD47" t="s">
         <v>37</v>
@@ -5663,13 +5678,13 @@
         <v>2025</v>
       </c>
       <c r="H48" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I48" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J48" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="P48">
         <v>0</v>
@@ -5684,16 +5699,16 @@
         <v>34</v>
       </c>
       <c r="Z48" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AA48" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AB48" t="s">
         <v>37</v>
       </c>
       <c r="AC48" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AD48" t="s">
         <v>37</v>
@@ -5722,13 +5737,13 @@
         <v>2025</v>
       </c>
       <c r="H49" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I49" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J49" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="P49">
         <v>0</v>
@@ -5743,16 +5758,16 @@
         <v>34</v>
       </c>
       <c r="Z49" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AA49" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="AB49" t="s">
         <v>37</v>
       </c>
       <c r="AC49" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="AD49" t="s">
         <v>37</v>
@@ -5781,13 +5796,13 @@
         <v>2025</v>
       </c>
       <c r="H50" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I50" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J50" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P50">
         <v>0</v>
@@ -5802,16 +5817,16 @@
         <v>34</v>
       </c>
       <c r="Z50" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AA50" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AB50" t="s">
         <v>37</v>
       </c>
       <c r="AC50" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="AD50" t="s">
         <v>37</v>
@@ -5840,13 +5855,13 @@
         <v>2025</v>
       </c>
       <c r="H51" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="I51" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J51" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P51">
         <v>0</v>
@@ -5861,16 +5876,16 @@
         <v>34</v>
       </c>
       <c r="Z51" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AA51" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AB51" t="s">
         <v>37</v>
       </c>
       <c r="AC51" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AD51" t="s">
         <v>37</v>
@@ -5899,13 +5914,13 @@
         <v>2025</v>
       </c>
       <c r="H52" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="I52" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J52" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P52">
         <v>0</v>
@@ -5920,16 +5935,16 @@
         <v>34</v>
       </c>
       <c r="Z52" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AA52" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="AB52" t="s">
         <v>37</v>
       </c>
       <c r="AC52" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AD52" t="s">
         <v>37</v>
@@ -5958,16 +5973,16 @@
         <v>2025</v>
       </c>
       <c r="H53" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I53" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J53" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K53" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="N53" t="s">
         <v>258</v>
@@ -5988,13 +6003,16 @@
         <v>34</v>
       </c>
       <c r="AA53" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AB53" t="s">
         <v>37</v>
       </c>
       <c r="AC53" t="s">
-        <v>342</v>
+        <v>344</v>
+      </c>
+      <c r="AD53" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="54" spans="1:30">
@@ -6020,10 +6038,10 @@
         <v>2025</v>
       </c>
       <c r="H54" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="I54" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="J54" t="s">
         <v>41</v>
@@ -6041,16 +6059,16 @@
         <v>34</v>
       </c>
       <c r="Z54" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="AA54" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="AB54" t="s">
         <v>37</v>
       </c>
       <c r="AC54" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="AD54" t="s">
         <v>37</v>
@@ -6079,13 +6097,13 @@
         <v>2025</v>
       </c>
       <c r="H55" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="I55" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="J55" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="P55">
         <v>0</v>
@@ -6100,16 +6118,16 @@
         <v>34</v>
       </c>
       <c r="Z55" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="AA55" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="AB55" t="s">
         <v>37</v>
       </c>
       <c r="AC55" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="AD55" t="s">
         <v>37</v>
@@ -6138,10 +6156,10 @@
         <v>2025</v>
       </c>
       <c r="H56" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="I56" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="J56" t="s">
         <v>41</v>
@@ -6159,16 +6177,16 @@
         <v>34</v>
       </c>
       <c r="Z56" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="AA56" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="AB56" t="s">
         <v>37</v>
       </c>
       <c r="AC56" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="AD56" t="s">
         <v>37</v>
@@ -6197,13 +6215,13 @@
         <v>2025</v>
       </c>
       <c r="H57" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="I57" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="J57" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="P57">
         <v>0</v>
@@ -6218,16 +6236,16 @@
         <v>34</v>
       </c>
       <c r="Z57" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="AA57" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="AB57" t="s">
         <v>37</v>
       </c>
       <c r="AC57" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="AD57" t="s">
         <v>37</v>
@@ -6256,13 +6274,13 @@
         <v>2025</v>
       </c>
       <c r="H58" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I58" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="J58" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="P58">
         <v>0</v>
@@ -6277,16 +6295,16 @@
         <v>34</v>
       </c>
       <c r="Z58" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="AA58" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="AB58" t="s">
         <v>37</v>
       </c>
       <c r="AC58" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="AD58" t="s">
         <v>37</v>
@@ -6315,13 +6333,13 @@
         <v>2025</v>
       </c>
       <c r="H59" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="I59" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="J59" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="P59">
         <v>0</v>
@@ -6336,16 +6354,16 @@
         <v>34</v>
       </c>
       <c r="Z59" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="AA59" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="AB59" t="s">
         <v>37</v>
       </c>
       <c r="AC59" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="AD59" t="s">
         <v>37</v>
@@ -6374,13 +6392,13 @@
         <v>2025</v>
       </c>
       <c r="H60" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="I60" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="J60" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="P60">
         <v>0</v>
@@ -6395,13 +6413,13 @@
         <v>34</v>
       </c>
       <c r="AA60" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="AB60" t="s">
         <v>37</v>
       </c>
       <c r="AC60" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="AD60" t="s">
         <v>37</v>
@@ -6430,10 +6448,10 @@
         <v>2025</v>
       </c>
       <c r="H61" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="I61" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="J61" t="s">
         <v>41</v>
@@ -6451,16 +6469,16 @@
         <v>34</v>
       </c>
       <c r="Z61" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="AA61" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="AB61" t="s">
         <v>37</v>
       </c>
       <c r="AC61" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="AD61" t="s">
         <v>37</v>
@@ -6489,13 +6507,13 @@
         <v>2025</v>
       </c>
       <c r="H62" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="I62" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="J62" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="P62">
         <v>0</v>
@@ -6510,16 +6528,16 @@
         <v>34</v>
       </c>
       <c r="Z62" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AA62" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AB62" t="s">
         <v>37</v>
       </c>
       <c r="AC62" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AD62" t="s">
         <v>37</v>
@@ -6548,13 +6566,13 @@
         <v>2025</v>
       </c>
       <c r="H63" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="I63" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="J63" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="P63">
         <v>0</v>
@@ -6569,16 +6587,16 @@
         <v>34</v>
       </c>
       <c r="Z63" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="AA63" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="AB63" t="s">
         <v>37</v>
       </c>
       <c r="AC63" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="AD63" t="s">
         <v>37</v>
@@ -6607,13 +6625,13 @@
         <v>2025</v>
       </c>
       <c r="H64" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="I64" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="J64" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="P64">
         <v>0</v>
@@ -6628,16 +6646,16 @@
         <v>34</v>
       </c>
       <c r="Z64" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="AA64" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AB64" t="s">
         <v>37</v>
       </c>
       <c r="AC64" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="AD64" t="s">
         <v>37</v>
@@ -6666,13 +6684,13 @@
         <v>2025</v>
       </c>
       <c r="H65" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="I65" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="J65" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="P65">
         <v>0</v>
@@ -6687,16 +6705,16 @@
         <v>34</v>
       </c>
       <c r="Z65" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="AA65" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="AB65" t="s">
         <v>37</v>
       </c>
       <c r="AC65" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="AD65" t="s">
         <v>37</v>
@@ -6725,13 +6743,13 @@
         <v>2025</v>
       </c>
       <c r="H66" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="I66" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="J66" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="P66">
         <v>0</v>
@@ -6746,16 +6764,16 @@
         <v>34</v>
       </c>
       <c r="Z66" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="AA66" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="AB66" t="s">
         <v>37</v>
       </c>
       <c r="AC66" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="AD66" t="s">
         <v>37</v>
@@ -6784,16 +6802,16 @@
         <v>2025</v>
       </c>
       <c r="H67" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="I67" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="J67" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="K67" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="N67" t="s">
         <v>91</v>
@@ -6805,7 +6823,7 @@
         <v>0</v>
       </c>
       <c r="Q67" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="S67">
         <v>0</v>
@@ -6817,16 +6835,19 @@
         <v>34</v>
       </c>
       <c r="Z67" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="AA67" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="AB67" t="s">
         <v>37</v>
       </c>
       <c r="AC67" t="s">
-        <v>423</v>
+        <v>426</v>
+      </c>
+      <c r="AD67" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="68" spans="1:30">
@@ -6852,13 +6873,13 @@
         <v>2025</v>
       </c>
       <c r="H68" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="I68" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="J68" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="P68">
         <v>0</v>
@@ -6873,16 +6894,16 @@
         <v>34</v>
       </c>
       <c r="Z68" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="AA68" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="AB68" t="s">
         <v>37</v>
       </c>
       <c r="AC68" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="AD68" t="s">
         <v>37</v>
@@ -6911,13 +6932,13 @@
         <v>2025</v>
       </c>
       <c r="H69" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="I69" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="J69" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="P69">
         <v>0</v>
@@ -6932,16 +6953,16 @@
         <v>34</v>
       </c>
       <c r="Z69" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="AA69" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="AB69" t="s">
         <v>37</v>
       </c>
       <c r="AC69" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="AD69" t="s">
         <v>37</v>
@@ -6970,13 +6991,13 @@
         <v>2025</v>
       </c>
       <c r="H70" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="I70" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="J70" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="P70">
         <v>0</v>
@@ -6991,16 +7012,16 @@
         <v>34</v>
       </c>
       <c r="Z70" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="AA70" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="AB70" t="s">
         <v>37</v>
       </c>
       <c r="AC70" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="AD70" t="s">
         <v>37</v>
@@ -7029,13 +7050,13 @@
         <v>2025</v>
       </c>
       <c r="H71" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="I71" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="J71" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="O71">
         <v>1</v>
@@ -7053,16 +7074,16 @@
         <v>34</v>
       </c>
       <c r="Z71" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="AA71" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="AB71" t="s">
         <v>37</v>
       </c>
       <c r="AC71" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="AD71" t="s">
         <v>37</v>
@@ -7091,13 +7112,13 @@
         <v>2025</v>
       </c>
       <c r="H72" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="I72" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="J72" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="P72">
         <v>0</v>
@@ -7112,16 +7133,16 @@
         <v>34</v>
       </c>
       <c r="Z72" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="AA72" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="AB72" t="s">
         <v>37</v>
       </c>
       <c r="AC72" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="AD72" t="s">
         <v>37</v>
@@ -7150,13 +7171,13 @@
         <v>2025</v>
       </c>
       <c r="H73" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="I73" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="J73" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="P73">
         <v>0</v>
@@ -7171,16 +7192,16 @@
         <v>34</v>
       </c>
       <c r="Z73" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="AA73" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="AB73" t="s">
         <v>37</v>
       </c>
       <c r="AC73" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="AD73" t="s">
         <v>37</v>
@@ -7209,16 +7230,16 @@
         <v>2025</v>
       </c>
       <c r="H74" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="I74" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="J74" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="K74" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="N74" t="s">
         <v>258</v>
@@ -7239,13 +7260,13 @@
         <v>34</v>
       </c>
       <c r="AA74" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="AB74" t="s">
         <v>37</v>
       </c>
       <c r="AC74" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="75" spans="1:30">
@@ -7271,13 +7292,13 @@
         <v>2025</v>
       </c>
       <c r="H75" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="I75" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="J75" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="P75">
         <v>0</v>
@@ -7292,16 +7313,16 @@
         <v>34</v>
       </c>
       <c r="Z75" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="AA75" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="AB75" t="s">
         <v>37</v>
       </c>
       <c r="AC75" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="AD75" t="s">
         <v>37</v>
@@ -7330,13 +7351,13 @@
         <v>2025</v>
       </c>
       <c r="H76" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="I76" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="J76" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="P76">
         <v>0</v>
@@ -7351,16 +7372,16 @@
         <v>34</v>
       </c>
       <c r="Z76" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="AA76" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="AB76" t="s">
         <v>37</v>
       </c>
       <c r="AC76" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="AD76" t="s">
         <v>37</v>
@@ -7389,13 +7410,13 @@
         <v>2025</v>
       </c>
       <c r="H77" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="I77" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="J77" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="P77">
         <v>0</v>
@@ -7410,16 +7431,16 @@
         <v>34</v>
       </c>
       <c r="Z77" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="AA77" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="AB77" t="s">
         <v>37</v>
       </c>
       <c r="AC77" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="AD77" t="s">
         <v>37</v>
@@ -7448,13 +7469,13 @@
         <v>2025</v>
       </c>
       <c r="H78" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="I78" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J78" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="P78">
         <v>0</v>
@@ -7469,16 +7490,16 @@
         <v>34</v>
       </c>
       <c r="Z78" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="AA78" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="AB78" t="s">
         <v>37</v>
       </c>
       <c r="AC78" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="AD78" t="s">
         <v>37</v>
@@ -7507,13 +7528,13 @@
         <v>2025</v>
       </c>
       <c r="H79" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="I79" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="J79" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="P79">
         <v>0</v>
@@ -7528,16 +7549,16 @@
         <v>34</v>
       </c>
       <c r="Z79" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="AA79" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="AB79" t="s">
         <v>37</v>
       </c>
       <c r="AC79" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="AD79" t="s">
         <v>37</v>
@@ -7566,13 +7587,13 @@
         <v>2025</v>
       </c>
       <c r="H80" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="I80" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="J80" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="P80">
         <v>0</v>
@@ -7587,16 +7608,16 @@
         <v>34</v>
       </c>
       <c r="Z80" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="AA80" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="AB80" t="s">
         <v>37</v>
       </c>
       <c r="AC80" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="AD80" t="s">
         <v>37</v>
@@ -7625,13 +7646,13 @@
         <v>2025</v>
       </c>
       <c r="H81" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="I81" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="J81" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="P81">
         <v>0</v>
@@ -7646,16 +7667,16 @@
         <v>34</v>
       </c>
       <c r="Z81" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="AA81" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="AB81" t="s">
         <v>37</v>
       </c>
       <c r="AC81" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="AD81" t="s">
         <v>37</v>
@@ -7684,13 +7705,13 @@
         <v>2025</v>
       </c>
       <c r="H82" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="I82" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="J82" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="P82">
         <v>0</v>
@@ -7705,16 +7726,16 @@
         <v>34</v>
       </c>
       <c r="Z82" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="AA82" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="AB82" t="s">
         <v>37</v>
       </c>
       <c r="AC82" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="AD82" t="s">
         <v>37</v>
@@ -7743,13 +7764,13 @@
         <v>2025</v>
       </c>
       <c r="H83" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="I83" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="J83" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="P83">
         <v>0</v>
@@ -7764,16 +7785,16 @@
         <v>34</v>
       </c>
       <c r="Z83" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="AA83" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="AB83" t="s">
         <v>37</v>
       </c>
       <c r="AC83" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="AD83" t="s">
         <v>37</v>
@@ -7802,13 +7823,13 @@
         <v>2025</v>
       </c>
       <c r="H84" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="I84" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="J84" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="P84">
         <v>0</v>
@@ -7823,16 +7844,16 @@
         <v>34</v>
       </c>
       <c r="Z84" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="AA84" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="AB84" t="s">
         <v>37</v>
       </c>
       <c r="AC84" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="AD84" t="s">
         <v>37</v>
@@ -7861,13 +7882,13 @@
         <v>2025</v>
       </c>
       <c r="H85" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="I85" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="J85" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="P85">
         <v>0</v>
@@ -7882,16 +7903,16 @@
         <v>34</v>
       </c>
       <c r="Z85" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="AA85" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="AB85" t="s">
         <v>37</v>
       </c>
       <c r="AC85" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="AD85" t="s">
         <v>37</v>
@@ -7920,13 +7941,13 @@
         <v>2025</v>
       </c>
       <c r="H86" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="I86" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="J86" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="P86">
         <v>0</v>
@@ -7941,16 +7962,16 @@
         <v>34</v>
       </c>
       <c r="Z86" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="AA86" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="AB86" t="s">
         <v>37</v>
       </c>
       <c r="AC86" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="AD86" t="s">
         <v>37</v>
@@ -7979,13 +8000,13 @@
         <v>2025</v>
       </c>
       <c r="H87" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="I87" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="J87" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="P87">
         <v>0</v>
@@ -8000,16 +8021,16 @@
         <v>34</v>
       </c>
       <c r="Z87" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="AA87" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="AB87" t="s">
         <v>37</v>
       </c>
       <c r="AC87" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="AD87" t="s">
         <v>37</v>
@@ -8038,13 +8059,13 @@
         <v>2025</v>
       </c>
       <c r="H88" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="I88" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J88" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="P88">
         <v>0</v>
@@ -8059,13 +8080,13 @@
         <v>34</v>
       </c>
       <c r="AA88" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="AB88" t="s">
         <v>37</v>
       </c>
       <c r="AC88" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="AD88" t="s">
         <v>37</v>
@@ -8094,10 +8115,10 @@
         <v>2025</v>
       </c>
       <c r="H89" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="I89" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="J89" t="s">
         <v>41</v>
@@ -8115,16 +8136,16 @@
         <v>34</v>
       </c>
       <c r="Z89" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="AA89" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="AB89" t="s">
         <v>37</v>
       </c>
       <c r="AC89" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="AD89" t="s">
         <v>37</v>
@@ -8153,13 +8174,13 @@
         <v>2025</v>
       </c>
       <c r="H90" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="I90" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="J90" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="P90">
         <v>0</v>
@@ -8174,16 +8195,16 @@
         <v>34</v>
       </c>
       <c r="Z90" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="AA90" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="AB90" t="s">
         <v>37</v>
       </c>
       <c r="AC90" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="AD90" t="s">
         <v>37</v>
@@ -8212,13 +8233,13 @@
         <v>2025</v>
       </c>
       <c r="H91" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="I91" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="J91" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="P91">
         <v>0</v>
@@ -8233,16 +8254,16 @@
         <v>34</v>
       </c>
       <c r="Z91" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="AA91" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="AB91" t="s">
         <v>37</v>
       </c>
       <c r="AC91" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="AD91" t="s">
         <v>37</v>
@@ -8271,13 +8292,13 @@
         <v>2025</v>
       </c>
       <c r="H92" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="I92" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J92" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="P92">
         <v>0</v>
@@ -8292,16 +8313,16 @@
         <v>34</v>
       </c>
       <c r="Z92" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="AA92" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="AB92" t="s">
         <v>37</v>
       </c>
       <c r="AC92" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="AD92" t="s">
         <v>37</v>
@@ -8330,13 +8351,13 @@
         <v>2025</v>
       </c>
       <c r="H93" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="I93" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="J93" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="P93">
         <v>0</v>
@@ -8351,16 +8372,16 @@
         <v>34</v>
       </c>
       <c r="Z93" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="AA93" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="AB93" t="s">
         <v>37</v>
       </c>
       <c r="AC93" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="AD93" t="s">
         <v>37</v>
@@ -8389,13 +8410,13 @@
         <v>2025</v>
       </c>
       <c r="H94" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="I94" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="J94" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="P94">
         <v>0</v>
@@ -8410,16 +8431,16 @@
         <v>34</v>
       </c>
       <c r="Z94" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="AA94" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="AB94" t="s">
         <v>37</v>
       </c>
       <c r="AC94" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="AD94" t="s">
         <v>37</v>
@@ -8448,25 +8469,25 @@
         <v>2025</v>
       </c>
       <c r="H95" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="I95" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="J95" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="K95" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="N95" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="P95">
         <v>0</v>
       </c>
       <c r="Q95" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="S95">
         <v>0</v>
@@ -8478,13 +8499,16 @@
         <v>34</v>
       </c>
       <c r="AA95" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="AB95" t="s">
         <v>37</v>
       </c>
       <c r="AC95" t="s">
-        <v>588</v>
+        <v>592</v>
+      </c>
+      <c r="AD95" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="96" spans="1:30">
@@ -8510,13 +8534,13 @@
         <v>2025</v>
       </c>
       <c r="H96" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="I96" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="J96" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="P96">
         <v>0</v>
@@ -8531,16 +8555,16 @@
         <v>34</v>
       </c>
       <c r="Z96" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="AA96" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="AB96" t="s">
         <v>37</v>
       </c>
       <c r="AC96" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="AD96" t="s">
         <v>37</v>
@@ -8569,13 +8593,13 @@
         <v>2025</v>
       </c>
       <c r="H97" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="I97" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="J97" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="P97">
         <v>0</v>
@@ -8590,16 +8614,16 @@
         <v>34</v>
       </c>
       <c r="Z97" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="AA97" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="AB97" t="s">
         <v>37</v>
       </c>
       <c r="AC97" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="AD97" t="s">
         <v>37</v>
@@ -8628,13 +8652,13 @@
         <v>2025</v>
       </c>
       <c r="H98" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="I98" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="J98" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="P98">
         <v>0</v>
@@ -8649,16 +8673,16 @@
         <v>34</v>
       </c>
       <c r="Z98" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="AA98" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="AB98" t="s">
         <v>37</v>
       </c>
       <c r="AC98" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="AD98" t="s">
         <v>37</v>
@@ -8687,10 +8711,10 @@
         <v>2025</v>
       </c>
       <c r="H99" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="I99" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="J99" t="s">
         <v>41</v>
@@ -8708,16 +8732,16 @@
         <v>34</v>
       </c>
       <c r="Z99" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="AA99" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="AB99" t="s">
         <v>37</v>
       </c>
       <c r="AC99" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="AD99" t="s">
         <v>37</v>
@@ -8746,13 +8770,13 @@
         <v>2025</v>
       </c>
       <c r="H100" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="I100" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="J100" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="P100">
         <v>0</v>
@@ -8767,16 +8791,16 @@
         <v>34</v>
       </c>
       <c r="Z100" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="AA100" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="AB100" t="s">
         <v>37</v>
       </c>
       <c r="AC100" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="AD100" t="s">
         <v>37</v>
@@ -8805,13 +8829,13 @@
         <v>2025</v>
       </c>
       <c r="H101" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="I101" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="J101" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="P101">
         <v>0</v>
@@ -8826,16 +8850,16 @@
         <v>34</v>
       </c>
       <c r="Z101" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="AA101" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="AB101" t="s">
         <v>37</v>
       </c>
       <c r="AC101" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="AD101" t="s">
         <v>37</v>
@@ -8864,16 +8888,16 @@
         <v>2025</v>
       </c>
       <c r="H102" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="I102" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="J102" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="K102" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="N102" t="s">
         <v>91</v>
@@ -8891,16 +8915,16 @@
         <v>34</v>
       </c>
       <c r="Z102" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="AA102" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="AB102" t="s">
         <v>37</v>
       </c>
       <c r="AC102" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
     </row>
     <row r="103" spans="1:30">
@@ -8926,13 +8950,13 @@
         <v>2025</v>
       </c>
       <c r="H103" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="I103" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="J103" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="P103">
         <v>0</v>
@@ -8947,16 +8971,16 @@
         <v>34</v>
       </c>
       <c r="Z103" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="AA103" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="AB103" t="s">
         <v>37</v>
       </c>
       <c r="AC103" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="AD103" t="s">
         <v>37</v>
@@ -8985,13 +9009,13 @@
         <v>2025</v>
       </c>
       <c r="H104" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="I104" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="J104" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="P104">
         <v>0</v>
@@ -9006,16 +9030,16 @@
         <v>34</v>
       </c>
       <c r="Z104" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="AA104" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="AB104" t="s">
         <v>37</v>
       </c>
       <c r="AC104" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="AD104" t="s">
         <v>37</v>
@@ -9044,13 +9068,13 @@
         <v>2025</v>
       </c>
       <c r="H105" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="I105" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="J105" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="P105">
         <v>0</v>
@@ -9065,16 +9089,16 @@
         <v>34</v>
       </c>
       <c r="Z105" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="AA105" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="AB105" t="s">
         <v>37</v>
       </c>
       <c r="AC105" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="AD105" t="s">
         <v>37</v>
@@ -9103,13 +9127,13 @@
         <v>2025</v>
       </c>
       <c r="H106" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="I106" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="J106" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="P106">
         <v>0</v>
@@ -9124,16 +9148,16 @@
         <v>34</v>
       </c>
       <c r="Z106" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="AA106" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="AB106" t="s">
         <v>37</v>
       </c>
       <c r="AC106" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="AD106" t="s">
         <v>37</v>
@@ -9162,13 +9186,13 @@
         <v>2025</v>
       </c>
       <c r="H107" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="I107" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="J107" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="P107">
         <v>0</v>
@@ -9183,16 +9207,16 @@
         <v>34</v>
       </c>
       <c r="Z107" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="AA107" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="AB107" t="s">
         <v>37</v>
       </c>
       <c r="AC107" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="AD107" t="s">
         <v>37</v>
@@ -9221,13 +9245,13 @@
         <v>2025</v>
       </c>
       <c r="H108" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="I108" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="J108" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="P108">
         <v>0</v>
@@ -9242,13 +9266,13 @@
         <v>34</v>
       </c>
       <c r="AA108" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="AB108" t="s">
         <v>37</v>
       </c>
       <c r="AC108" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="AD108" t="s">
         <v>37</v>
@@ -9277,10 +9301,10 @@
         <v>2025</v>
       </c>
       <c r="H109" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="I109" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="J109" t="s">
         <v>173</v>
@@ -9304,16 +9328,16 @@
         <v>34</v>
       </c>
       <c r="Z109" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="AA109" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="AB109" t="s">
         <v>37</v>
       </c>
       <c r="AC109" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
     </row>
     <row r="110" spans="1:30">
@@ -9339,13 +9363,13 @@
         <v>2025</v>
       </c>
       <c r="H110" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="I110" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="J110" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="P110">
         <v>0</v>
@@ -9360,16 +9384,16 @@
         <v>34</v>
       </c>
       <c r="Z110" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="AA110" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="AB110" t="s">
         <v>37</v>
       </c>
       <c r="AC110" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="AD110" t="s">
         <v>37</v>
@@ -9398,13 +9422,13 @@
         <v>2025</v>
       </c>
       <c r="H111" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="I111" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="J111" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="P111">
         <v>0</v>
@@ -9419,16 +9443,16 @@
         <v>34</v>
       </c>
       <c r="Z111" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="AA111" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="AB111" t="s">
         <v>37</v>
       </c>
       <c r="AC111" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="AD111" t="s">
         <v>37</v>
@@ -9457,13 +9481,13 @@
         <v>2025</v>
       </c>
       <c r="H112" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="I112" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="J112" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="P112">
         <v>0</v>
@@ -9478,16 +9502,16 @@
         <v>34</v>
       </c>
       <c r="Z112" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="AA112" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="AB112" t="s">
         <v>37</v>
       </c>
       <c r="AC112" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="AD112" t="s">
         <v>37</v>
@@ -9516,13 +9540,13 @@
         <v>2025</v>
       </c>
       <c r="H113" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="I113" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="J113" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="P113">
         <v>0</v>
@@ -9537,16 +9561,16 @@
         <v>34</v>
       </c>
       <c r="Z113" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="AA113" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="AB113" t="s">
         <v>37</v>
       </c>
       <c r="AC113" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="AD113" t="s">
         <v>37</v>
@@ -9575,13 +9599,13 @@
         <v>2025</v>
       </c>
       <c r="H114" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="I114" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="J114" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="P114">
         <v>0</v>
@@ -9596,16 +9620,16 @@
         <v>34</v>
       </c>
       <c r="Z114" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="AA114" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="AB114" t="s">
         <v>37</v>
       </c>
       <c r="AC114" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="AD114" t="s">
         <v>37</v>
@@ -9634,13 +9658,13 @@
         <v>2025</v>
       </c>
       <c r="H115" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="I115" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="J115" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="P115">
         <v>0</v>
@@ -9655,16 +9679,16 @@
         <v>34</v>
       </c>
       <c r="Z115" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="AA115" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="AB115" t="s">
         <v>37</v>
       </c>
       <c r="AC115" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="AD115" t="s">
         <v>37</v>
@@ -9693,16 +9717,16 @@
         <v>2025</v>
       </c>
       <c r="H116" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="I116" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="J116" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="K116" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="P116">
         <v>0</v>
@@ -9717,16 +9741,16 @@
         <v>34</v>
       </c>
       <c r="Z116" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="AA116" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="AB116" t="s">
         <v>37</v>
       </c>
       <c r="AC116" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
     </row>
     <row r="117" spans="1:30">
@@ -9752,13 +9776,13 @@
         <v>2025</v>
       </c>
       <c r="H117" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="I117" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="J117" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="P117">
         <v>0</v>
@@ -9773,16 +9797,16 @@
         <v>34</v>
       </c>
       <c r="Z117" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="AA117" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="AB117" t="s">
         <v>37</v>
       </c>
       <c r="AC117" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="AD117" t="s">
         <v>37</v>
@@ -9811,16 +9835,16 @@
         <v>2025</v>
       </c>
       <c r="H118" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="I118" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="J118" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="K118" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="P118">
         <v>0</v>
@@ -9835,13 +9859,13 @@
         <v>34</v>
       </c>
       <c r="AA118" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="AB118" t="s">
         <v>37</v>
       </c>
       <c r="AC118" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
     </row>
     <row r="119" spans="1:30">
@@ -9867,13 +9891,13 @@
         <v>2025</v>
       </c>
       <c r="H119" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="I119" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="J119" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="P119">
         <v>0</v>
@@ -9888,16 +9912,16 @@
         <v>34</v>
       </c>
       <c r="Z119" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="AA119" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="AB119" t="s">
         <v>37</v>
       </c>
       <c r="AC119" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="AD119" t="s">
         <v>37</v>
@@ -9926,13 +9950,13 @@
         <v>2025</v>
       </c>
       <c r="H120" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="I120" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="J120" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="P120">
         <v>0</v>
@@ -9947,16 +9971,16 @@
         <v>34</v>
       </c>
       <c r="Z120" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="AA120" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="AB120" t="s">
         <v>37</v>
       </c>
       <c r="AC120" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="AD120" t="s">
         <v>37</v>
@@ -9985,13 +10009,13 @@
         <v>2025</v>
       </c>
       <c r="H121" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="I121" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="J121" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="P121">
         <v>0</v>
@@ -10006,16 +10030,16 @@
         <v>34</v>
       </c>
       <c r="Z121" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="AA121" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="AB121" t="s">
         <v>37</v>
       </c>
       <c r="AC121" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
     </row>
     <row r="122" spans="1:30">
@@ -10041,13 +10065,13 @@
         <v>2025</v>
       </c>
       <c r="H122" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="I122" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="J122" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="P122">
         <v>0</v>
@@ -10062,16 +10086,16 @@
         <v>34</v>
       </c>
       <c r="Z122" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="AA122" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="AB122" t="s">
         <v>37</v>
       </c>
       <c r="AC122" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
     </row>
     <row r="123" spans="1:30">
@@ -10097,10 +10121,10 @@
         <v>2025</v>
       </c>
       <c r="H123" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="I123" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="P123">
         <v>0</v>
@@ -10115,16 +10139,16 @@
         <v>34</v>
       </c>
       <c r="Z123" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="AA123" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="AB123" t="s">
         <v>37</v>
       </c>
       <c r="AC123" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="AD123" t="s">
         <v>37</v>
@@ -10153,13 +10177,13 @@
         <v>2025</v>
       </c>
       <c r="H124" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="I124" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="J124" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="P124">
         <v>0</v>
@@ -10174,16 +10198,16 @@
         <v>34</v>
       </c>
       <c r="Z124" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="AA124" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="AB124" t="s">
         <v>37</v>
       </c>
       <c r="AC124" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="125" spans="1:30">
@@ -10209,13 +10233,13 @@
         <v>2025</v>
       </c>
       <c r="H125" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="I125" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="J125" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="P125">
         <v>0</v>
@@ -10230,16 +10254,16 @@
         <v>34</v>
       </c>
       <c r="Z125" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="AA125" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="AB125" t="s">
         <v>37</v>
       </c>
       <c r="AC125" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="AD125" t="s">
         <v>37</v>
@@ -10268,16 +10292,16 @@
         <v>2025</v>
       </c>
       <c r="H126" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="I126" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="J126" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="K126" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="N126" t="s">
         <v>91</v>
@@ -10286,13 +10310,13 @@
         <v>34</v>
       </c>
       <c r="AA126" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="AB126" t="s">
         <v>37</v>
       </c>
       <c r="AC126" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="AD126" t="s">
         <v>37</v>
@@ -10321,10 +10345,10 @@
         <v>2025</v>
       </c>
       <c r="H127" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="I127" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="P127">
         <v>0</v>
@@ -10339,13 +10363,13 @@
         <v>34</v>
       </c>
       <c r="AA127" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="AB127" t="s">
         <v>37</v>
       </c>
       <c r="AC127" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
     </row>
     <row r="128" spans="1:30">
@@ -10371,16 +10395,16 @@
         <v>2025</v>
       </c>
       <c r="H128" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="I128" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="J128" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="K128" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="L128">
         <v>4</v>
@@ -10407,16 +10431,16 @@
         <v>34</v>
       </c>
       <c r="Z128" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="AA128" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="AB128" t="s">
         <v>37</v>
       </c>
       <c r="AC128" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="AD128" t="s">
         <v>37</v>
@@ -10445,16 +10469,16 @@
         <v>2025</v>
       </c>
       <c r="H129" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="I129" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="J129" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="K129" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="L129">
         <v>4</v>
@@ -10478,16 +10502,16 @@
         <v>34</v>
       </c>
       <c r="Z129" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="AA129" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="AB129" t="s">
         <v>37</v>
       </c>
       <c r="AC129" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="AD129" t="s">
         <v>37</v>
@@ -10516,16 +10540,16 @@
         <v>2025</v>
       </c>
       <c r="H130" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="I130" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="J130" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="K130" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="L130">
         <v>2</v>
@@ -10534,7 +10558,7 @@
         <v>2</v>
       </c>
       <c r="N130" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="P130">
         <v>0</v>
@@ -10549,13 +10573,13 @@
         <v>34</v>
       </c>
       <c r="AA130" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="AB130" t="s">
         <v>37</v>
       </c>
       <c r="AC130" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AD130" t="s">
         <v>37</v>
@@ -10584,16 +10608,16 @@
         <v>2025</v>
       </c>
       <c r="H131" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="I131" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="J131" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="K131" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="L131">
         <v>2</v>
@@ -10602,7 +10626,7 @@
         <v>2</v>
       </c>
       <c r="N131" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="O131">
         <v>7</v>
@@ -10620,16 +10644,16 @@
         <v>34</v>
       </c>
       <c r="Z131" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="AA131" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="AB131" t="s">
         <v>37</v>
       </c>
       <c r="AC131" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
     <row r="132" spans="1:30">
@@ -10655,16 +10679,16 @@
         <v>2025</v>
       </c>
       <c r="H132" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="I132" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="J132" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="K132" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="L132">
         <v>3</v>
@@ -10673,7 +10697,7 @@
         <v>4</v>
       </c>
       <c r="N132" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="P132">
         <v>0</v>
@@ -10688,13 +10712,13 @@
         <v>34</v>
       </c>
       <c r="AA132" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="AB132" t="s">
         <v>37</v>
       </c>
       <c r="AC132" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
     </row>
     <row r="133" spans="1:30">
@@ -10720,16 +10744,16 @@
         <v>2025</v>
       </c>
       <c r="H133" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="I133" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="J133" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="K133" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="L133">
         <v>1</v>
@@ -10738,7 +10762,7 @@
         <v>1</v>
       </c>
       <c r="N133" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="O133">
         <v>5</v>
@@ -10756,13 +10780,13 @@
         <v>34</v>
       </c>
       <c r="AA133" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="AB133" t="s">
         <v>37</v>
       </c>
       <c r="AC133" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
     </row>
     <row r="134" spans="1:30">
@@ -10788,16 +10812,16 @@
         <v>2025</v>
       </c>
       <c r="H134" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="I134" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="J134" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="K134" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="L134">
         <v>1</v>
@@ -10824,16 +10848,16 @@
         <v>34</v>
       </c>
       <c r="Z134" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="AA134" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="AB134" t="s">
         <v>37</v>
       </c>
       <c r="AC134" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="AD134" t="s">
         <v>37</v>
@@ -10862,16 +10886,16 @@
         <v>2025</v>
       </c>
       <c r="H135" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="I135" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="J135" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="K135" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="L135">
         <v>3</v>
@@ -10880,7 +10904,7 @@
         <v>4</v>
       </c>
       <c r="N135" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="O135">
         <v>8</v>
@@ -10898,13 +10922,13 @@
         <v>34</v>
       </c>
       <c r="AA135" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="AB135" t="s">
         <v>37</v>
       </c>
       <c r="AC135" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
     </row>
     <row r="136" spans="1:30">
@@ -10930,16 +10954,16 @@
         <v>2025</v>
       </c>
       <c r="H136" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="I136" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="J136" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="K136" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="L136">
         <v>2</v>
@@ -10966,16 +10990,16 @@
         <v>34</v>
       </c>
       <c r="Z136" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="AA136" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
       <c r="AB136" t="s">
         <v>37</v>
       </c>
       <c r="AC136" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="AD136" t="s">
         <v>37</v>

</xml_diff>